<commit_message>
First big prep disag (no general)
</commit_message>
<xml_diff>
--- a/Submissions/Scale summary.xlsx
+++ b/Submissions/Scale summary.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adenooy/Library/CloudStorage/OneDrive-Personal/AMC/HIV Prioritization tool/HIV_prioritization_tool/Submissions/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/Submissions/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{5759D780-3FB7-1346-8B5F-890D1F20736E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5020" yWindow="2860" windowWidth="27240" windowHeight="14940" xr2:uid="{18B8B138-094E-AE42-8954-D756218EA68A}"/>
+    <workbookView xWindow="1560" yWindow="1780" windowWidth="27240" windowHeight="14940" xr2:uid="{18B8B138-094E-AE42-8954-D756218EA68A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -264,45 +264,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -312,12 +297,21 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -334,10 +328,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -657,7 +647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BE5D1EB-8B7D-694B-AD6A-EE173EAA4F7D}">
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.1640625" bestFit="1" customWidth="1"/>
@@ -669,580 +659,548 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="11" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="14" t="s">
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
+      <c r="H1" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="M1" s="1"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="28"/>
+      <c r="L1" s="28"/>
+      <c r="M1" s="28"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A2" s="2"/>
-      <c r="B2" s="6" t="s">
+      <c r="A2" s="25"/>
+      <c r="B2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="15" t="s">
+      <c r="I2" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="15" t="s">
+      <c r="J2" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="12"/>
-      <c r="L2" s="12"/>
-      <c r="M2" s="12"/>
+      <c r="K2" s="7"/>
+      <c r="L2" s="7"/>
+      <c r="M2" s="7"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A3" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="7">
-        <v>0</v>
-      </c>
-      <c r="C3" s="7">
-        <v>0</v>
-      </c>
-      <c r="D3" s="8">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>0</v>
+      </c>
+      <c r="D3" s="4">
         <v>30762</v>
       </c>
-      <c r="E3" s="13">
+      <c r="E3" s="8">
         <f>ROUND(1.15*B3,0)</f>
         <v>0</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="8">
         <f t="shared" ref="F3:G3" si="0">ROUND(1.15*C3,0)</f>
         <v>0</v>
       </c>
-      <c r="G3" s="32">
+      <c r="G3" s="19">
         <f t="shared" si="0"/>
         <v>35376</v>
       </c>
-      <c r="H3" s="33">
+      <c r="H3" s="20">
         <f>ROUND(0.85*B3,0)</f>
         <v>0</v>
       </c>
-      <c r="I3" s="33">
+      <c r="I3" s="20">
         <f t="shared" ref="I3:J3" si="1">ROUND(0.85*C3,0)</f>
         <v>0</v>
       </c>
-      <c r="J3" s="33">
+      <c r="J3" s="20">
         <f t="shared" si="1"/>
         <v>26148</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="5">
         <v>11237387</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="6">
         <v>3671497</v>
       </c>
-      <c r="D4" s="8">
+      <c r="D4" s="4">
         <v>3569803</v>
       </c>
-      <c r="E4" s="32">
+      <c r="E4" s="19">
         <f t="shared" ref="E4:E9" si="2">ROUND(1.15*B4,0)</f>
         <v>12922995</v>
       </c>
-      <c r="F4" s="32">
+      <c r="F4" s="19">
         <f t="shared" ref="F4:F9" si="3">ROUND(1.15*C4,0)</f>
         <v>4222222</v>
       </c>
-      <c r="G4" s="32">
+      <c r="G4" s="19">
         <f t="shared" ref="G4:G9" si="4">ROUND(1.15*D4,0)</f>
         <v>4105273</v>
       </c>
-      <c r="H4" s="33">
+      <c r="H4" s="20">
         <f t="shared" ref="H4:H9" si="5">ROUND(0.85*B4,0)</f>
         <v>9551779</v>
       </c>
-      <c r="I4" s="33">
+      <c r="I4" s="20">
         <f t="shared" ref="I4:I9" si="6">ROUND(0.85*C4,0)</f>
         <v>3120772</v>
       </c>
-      <c r="J4" s="33">
+      <c r="J4" s="20">
         <f t="shared" ref="J4:J9" si="7">ROUND(0.85*D4,0)</f>
         <v>3034333</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="5">
         <v>630566</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="6">
         <v>291365</v>
       </c>
-      <c r="D5" s="8">
+      <c r="D5" s="4">
         <v>129230</v>
       </c>
-      <c r="E5" s="32">
+      <c r="E5" s="19">
         <f t="shared" si="2"/>
         <v>725151</v>
       </c>
-      <c r="F5" s="32">
+      <c r="F5" s="19">
         <f t="shared" si="3"/>
         <v>335070</v>
       </c>
-      <c r="G5" s="32">
+      <c r="G5" s="19">
         <f t="shared" si="4"/>
         <v>148615</v>
       </c>
-      <c r="H5" s="33">
+      <c r="H5" s="20">
         <f t="shared" si="5"/>
         <v>535981</v>
       </c>
-      <c r="I5" s="33">
+      <c r="I5" s="20">
         <f t="shared" si="6"/>
         <v>247660</v>
       </c>
-      <c r="J5" s="33">
+      <c r="J5" s="20">
         <f t="shared" si="7"/>
         <v>109846</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="5">
         <v>1064884</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="6">
         <v>516869</v>
       </c>
-      <c r="D6" s="8">
+      <c r="D6" s="4">
         <v>129013</v>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="19">
         <f t="shared" si="2"/>
         <v>1224617</v>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="19">
         <f t="shared" si="3"/>
         <v>594399</v>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="19">
         <f t="shared" si="4"/>
         <v>148365</v>
       </c>
-      <c r="H6" s="33">
+      <c r="H6" s="20">
         <f t="shared" si="5"/>
         <v>905151</v>
       </c>
-      <c r="I6" s="33">
+      <c r="I6" s="20">
         <f t="shared" si="6"/>
         <v>439339</v>
       </c>
-      <c r="J6" s="33">
+      <c r="J6" s="20">
         <f t="shared" si="7"/>
         <v>109661</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="5">
         <v>222182</v>
       </c>
-      <c r="C7" s="10">
-        <v>0</v>
-      </c>
-      <c r="D7" s="8">
+      <c r="C7" s="6">
+        <v>0</v>
+      </c>
+      <c r="D7" s="4">
         <v>513183</v>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="19">
         <f t="shared" si="2"/>
         <v>255509</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="19">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="19">
         <f t="shared" si="4"/>
         <v>590160</v>
       </c>
-      <c r="H7" s="33">
+      <c r="H7" s="20">
         <f t="shared" si="5"/>
         <v>188855</v>
       </c>
-      <c r="I7" s="33">
+      <c r="I7" s="20">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J7" s="33">
+      <c r="J7" s="20">
         <f t="shared" si="7"/>
         <v>436206</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="9">
-        <v>0</v>
-      </c>
-      <c r="C8" s="10">
-        <v>0</v>
-      </c>
-      <c r="D8" s="8">
+      <c r="B8" s="5">
+        <v>0</v>
+      </c>
+      <c r="C8" s="6">
+        <v>0</v>
+      </c>
+      <c r="D8" s="4">
         <v>1741863</v>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="19">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="19">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="19">
         <f t="shared" si="4"/>
         <v>2003142</v>
       </c>
-      <c r="H8" s="33">
+      <c r="H8" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I8" s="33">
+      <c r="I8" s="20">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J8" s="33">
+      <c r="J8" s="20">
         <f t="shared" si="7"/>
         <v>1480584</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A9" s="4" t="s">
+      <c r="A9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="5">
         <v>1322885</v>
       </c>
-      <c r="C9" s="10">
-        <v>0</v>
-      </c>
-      <c r="D9" s="8">
+      <c r="C9" s="6">
+        <v>0</v>
+      </c>
+      <c r="D9" s="4">
         <v>60432</v>
       </c>
-      <c r="E9" s="32">
+      <c r="E9" s="19">
         <f t="shared" si="2"/>
         <v>1521318</v>
       </c>
-      <c r="F9" s="32">
+      <c r="F9" s="19">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="19">
         <f t="shared" si="4"/>
         <v>69497</v>
       </c>
-      <c r="H9" s="33">
+      <c r="H9" s="20">
         <f t="shared" si="5"/>
         <v>1124452</v>
       </c>
-      <c r="I9" s="33">
+      <c r="I9" s="20">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="J9" s="33">
+      <c r="J9" s="20">
         <f t="shared" si="7"/>
         <v>51367</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-    </row>
-    <row r="11" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-    </row>
+    <row r="11" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="12" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
-      <c r="F12" s="28"/>
-      <c r="G12" s="26" t="s">
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="H12" s="27"/>
-      <c r="I12" s="27"/>
-      <c r="J12" s="27"/>
-      <c r="K12" s="28"/>
-      <c r="L12" s="26" t="s">
+      <c r="H12" s="22"/>
+      <c r="I12" s="22"/>
+      <c r="J12" s="22"/>
+      <c r="K12" s="23"/>
+      <c r="L12" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27"/>
-      <c r="O12" s="27"/>
-      <c r="P12" s="28"/>
+      <c r="M12" s="22"/>
+      <c r="N12" s="22"/>
+      <c r="O12" s="22"/>
+      <c r="P12" s="23"/>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="B13" s="29" t="s">
+      <c r="B13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="E13" s="30" t="s">
+      <c r="E13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="31" t="s">
+      <c r="F13" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="29" t="s">
+      <c r="G13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="H13" s="30" t="s">
+      <c r="H13" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="I13" s="30" t="s">
+      <c r="I13" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="J13" s="30" t="s">
+      <c r="J13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="K13" s="31" t="s">
+      <c r="K13" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="L13" s="29" t="s">
+      <c r="L13" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="M13" s="30" t="s">
+      <c r="M13" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="N13" s="30" t="s">
+      <c r="N13" s="17" t="s">
         <v>16</v>
       </c>
-      <c r="O13" s="30" t="s">
+      <c r="O13" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="P13" s="31" t="s">
+      <c r="P13" s="18" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="11">
         <v>90.5</v>
       </c>
-      <c r="C14" s="3">
+      <c r="C14">
         <v>95.3</v>
       </c>
-      <c r="D14" s="3">
+      <c r="D14">
         <v>92.6</v>
       </c>
-      <c r="E14" s="34">
+      <c r="E14">
         <v>44391</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="12">
         <v>91525</v>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="11">
         <v>95.6</v>
       </c>
-      <c r="H14" s="34">
+      <c r="H14">
         <v>97.8</v>
       </c>
-      <c r="I14" s="34">
+      <c r="I14">
         <v>98</v>
       </c>
-      <c r="J14" s="34">
+      <c r="J14">
         <v>16336</v>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="12">
         <v>30400</v>
       </c>
-      <c r="L14" s="21">
+      <c r="L14" s="11">
         <v>96.4</v>
       </c>
-      <c r="M14" s="3">
+      <c r="M14">
         <v>96.1</v>
       </c>
-      <c r="N14" s="3">
+      <c r="N14">
         <v>95.9</v>
       </c>
-      <c r="O14" s="34">
+      <c r="O14">
         <v>13450</v>
       </c>
-      <c r="P14" s="22">
+      <c r="P14" s="12">
         <v>11757</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.2">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="11">
         <v>0.5</v>
       </c>
-      <c r="C15" s="3">
-        <v>0</v>
-      </c>
-      <c r="D15" s="3">
-        <v>0</v>
-      </c>
-      <c r="E15" s="34">
+      <c r="C15">
+        <v>0</v>
+      </c>
+      <c r="D15">
+        <v>0</v>
+      </c>
+      <c r="E15">
         <v>-0.5</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="12">
         <v>-1.7</v>
       </c>
-      <c r="G15" s="21">
+      <c r="G15" s="11">
         <v>0.3</v>
       </c>
-      <c r="H15" s="34">
-        <v>0</v>
-      </c>
-      <c r="I15" s="34">
-        <v>0</v>
-      </c>
-      <c r="J15" s="34">
+      <c r="H15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
         <v>-0.5</v>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="12">
         <v>-2.8</v>
       </c>
-      <c r="L15" s="21">
+      <c r="L15" s="11">
         <v>0.2</v>
       </c>
-      <c r="M15" s="3">
-        <v>0</v>
-      </c>
-      <c r="N15" s="3">
+      <c r="M15">
+        <v>0</v>
+      </c>
+      <c r="N15">
         <v>0.1</v>
       </c>
-      <c r="O15" s="34">
+      <c r="O15">
         <v>-0.3</v>
       </c>
-      <c r="P15" s="22">
+      <c r="P15" s="12">
         <v>-1.1000000000000001</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
+      <c r="A16" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B16" s="23">
+      <c r="B16" s="13">
         <v>-0.6</v>
       </c>
-      <c r="C16" s="24">
-        <v>0</v>
-      </c>
-      <c r="D16" s="24">
-        <v>0</v>
-      </c>
-      <c r="E16" s="24">
+      <c r="C16" s="14">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14">
+        <v>0</v>
+      </c>
+      <c r="E16" s="14">
         <v>0.5</v>
       </c>
-      <c r="F16" s="25">
+      <c r="F16" s="15">
         <v>1.7</v>
       </c>
-      <c r="G16" s="23">
+      <c r="G16" s="13">
         <v>-0.4</v>
       </c>
-      <c r="H16" s="24">
-        <v>0</v>
-      </c>
-      <c r="I16" s="24">
-        <v>0</v>
-      </c>
-      <c r="J16" s="24">
+      <c r="H16" s="14">
+        <v>0</v>
+      </c>
+      <c r="I16" s="14">
+        <v>0</v>
+      </c>
+      <c r="J16" s="14">
         <v>0.5</v>
       </c>
-      <c r="K16" s="25">
+      <c r="K16" s="15">
         <v>2.8</v>
       </c>
-      <c r="L16" s="23">
+      <c r="L16" s="13">
         <f>-0.5</f>
         <v>-0.5</v>
       </c>
-      <c r="M16" s="24">
-        <v>0</v>
-      </c>
-      <c r="N16" s="24">
-        <v>0</v>
-      </c>
-      <c r="O16" s="24">
+      <c r="M16" s="14">
+        <v>0</v>
+      </c>
+      <c r="N16" s="14">
+        <v>0</v>
+      </c>
+      <c r="O16" s="14">
         <v>0.5</v>
       </c>
-      <c r="P16" s="25">
+      <c r="P16" s="15">
         <v>2.2999999999999998</v>
       </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="19"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="19"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="19"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="20"/>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="20"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>